<commit_message>
invoicing: clear stale hardcoded 2.05.x amounts in JBCON cover template
Cover sheet C28/C29 shipped with leftover values ($9,318.30 / $1,494.27) the
generator never cleared, inflating 'This Invoice' to $15,103.70. Blanked them so
the cover foots to the actual billed total.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/invoicing/templates/JBCON_template.xlsx
+++ b/invoicing/templates/JBCON_template.xlsx
@@ -4156,9 +4156,7 @@
       <c r="B28" s="125">
         <v>0</v>
       </c>
-      <c r="C28" s="125">
-        <v>9318.2999999999993</v>
-      </c>
+      <c r="C28"/>
       <c r="D28" s="125">
         <f t="shared" si="0"/>
         <v>9318.2999999999993</v>
@@ -4178,9 +4176,7 @@
       <c r="B29" s="125">
         <v>0</v>
       </c>
-      <c r="C29" s="125">
-        <v>1494.27</v>
-      </c>
+      <c r="C29"/>
       <c r="D29" s="125">
         <f t="shared" si="0"/>
         <v>1494.27</v>

</xml_diff>